<commit_message>
Improve COE uploads, templates, and portal UX for staff and students.
Sync student profile edits across related tables, expand marks template samples, parse library Returned/Not Returned on upload, hide login emails in headers, and refine admin queue sorting labels.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/marks_template_final.xlsx
+++ b/public/marks_template_final.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AL2"/>
+  <dimension ref="A1:AK17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -511,9 +511,6 @@
       <c r="AK1" t="str">
         <v>Grade Points</v>
       </c>
-      <c r="AL1" t="str">
-        <v>Image Path</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -535,7 +532,7 @@
         <v>SCHOOL OF SCIENCES</v>
       </c>
       <c r="G2" t="str">
-        <v>Bachelor of Science Food Science and Technology, Biochemistry and Microbiology</v>
+        <v>Bachelor of Science Food Science and Technology</v>
       </c>
       <c r="H2" t="str">
         <v>BSFT</v>
@@ -550,10 +547,10 @@
         <v>2026-05-04</v>
       </c>
       <c r="L2" t="str">
-        <v>VI</v>
+        <v>IV</v>
       </c>
       <c r="M2" t="str">
-        <v>GCBSFT00021</v>
+        <v>GCBSFT00001</v>
       </c>
       <c r="N2" t="str">
         <v>CORE COURSE</v>
@@ -565,10 +562,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="str">
-        <v>23BSFT101T1</v>
+        <v>SUB101</v>
       </c>
       <c r="R2" t="str">
-        <v>Food Chemistry</v>
+        <v>Introduction to Subject One</v>
       </c>
       <c r="S2">
         <v>4</v>
@@ -589,7 +586,7 @@
         <v>0</v>
       </c>
       <c r="Y2">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -607,7 +604,7 @@
         <v>0</v>
       </c>
       <c r="AE2">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="AF2">
         <v>0</v>
@@ -627,13 +624,1705 @@
       <c r="AK2">
         <v>8</v>
       </c>
-      <c r="AL2" t="str">
-        <v>23BSFT101.jpg</v>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>23bsft101@gcu.edu.in</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Abigail Albert Anbudurai</v>
+      </c>
+      <c r="D3" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F3" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H3" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I3" t="str">
+        <v>23BSFT101</v>
+      </c>
+      <c r="J3" t="str">
+        <v>April - 2026</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L3" t="str">
+        <v>IV</v>
+      </c>
+      <c r="M3" t="str">
+        <v>GCBSFT00001</v>
+      </c>
+      <c r="N3" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O3" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P3">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>SUB102</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Introduction to Subject Two</v>
+      </c>
+      <c r="S3">
+        <v>4</v>
+      </c>
+      <c r="T3">
+        <v>4</v>
+      </c>
+      <c r="U3">
+        <v>40</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>16</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>35.2</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>60</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
+      </c>
+      <c r="AC3">
+        <v>24</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>52.8</v>
+      </c>
+      <c r="AF3">
+        <v>0</v>
+      </c>
+      <c r="AG3">
+        <v>100</v>
+      </c>
+      <c r="AH3">
+        <v>0</v>
+      </c>
+      <c r="AI3" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ3" t="str">
+        <v>A+</v>
+      </c>
+      <c r="AK3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>23bsft101@gcu.edu.in</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Abigail Albert Anbudurai</v>
+      </c>
+      <c r="D4" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F4" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H4" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I4" t="str">
+        <v>23BSFT101</v>
+      </c>
+      <c r="J4" t="str">
+        <v>April - 2026</v>
+      </c>
+      <c r="K4" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L4" t="str">
+        <v>IV</v>
+      </c>
+      <c r="M4" t="str">
+        <v>GCBSFT00001</v>
+      </c>
+      <c r="N4" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O4" t="str">
+        <v>PRACTICAL</v>
+      </c>
+      <c r="P4">
+        <v>1</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>SUB103P</v>
+      </c>
+      <c r="R4" t="str">
+        <v>Practical Lab One</v>
+      </c>
+      <c r="S4">
+        <v>4</v>
+      </c>
+      <c r="T4">
+        <v>4</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>40</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>16</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>38</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>60</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>24</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
+      <c r="AF4">
+        <v>57</v>
+      </c>
+      <c r="AG4">
+        <v>100</v>
+      </c>
+      <c r="AH4">
+        <v>0</v>
+      </c>
+      <c r="AI4" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ4" t="str">
+        <v>O</v>
+      </c>
+      <c r="AK4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>23bsft101@gcu.edu.in</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Abigail Albert Anbudurai</v>
+      </c>
+      <c r="D5" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F5" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H5" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I5" t="str">
+        <v>23BSFT101</v>
+      </c>
+      <c r="J5" t="str">
+        <v>April - 2026</v>
+      </c>
+      <c r="K5" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L5" t="str">
+        <v>IV</v>
+      </c>
+      <c r="M5" t="str">
+        <v>GCBSFT00001</v>
+      </c>
+      <c r="N5" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O5" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P5">
+        <v>1</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>SUB104</v>
+      </c>
+      <c r="R5" t="str">
+        <v>Advanced Subject Four</v>
+      </c>
+      <c r="S5">
+        <v>4</v>
+      </c>
+      <c r="T5">
+        <v>4</v>
+      </c>
+      <c r="U5">
+        <v>40</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>16</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>27.200000000000003</v>
+      </c>
+      <c r="Z5">
+        <v>0</v>
+      </c>
+      <c r="AA5">
+        <v>60</v>
+      </c>
+      <c r="AB5">
+        <v>0</v>
+      </c>
+      <c r="AC5">
+        <v>24</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+      <c r="AE5">
+        <v>40.8</v>
+      </c>
+      <c r="AF5">
+        <v>0</v>
+      </c>
+      <c r="AG5">
+        <v>100</v>
+      </c>
+      <c r="AH5">
+        <v>0</v>
+      </c>
+      <c r="AI5" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ5" t="str">
+        <v>B+</v>
+      </c>
+      <c r="AK5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>23bsft101@gcu.edu.in</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Abigail Albert Anbudurai</v>
+      </c>
+      <c r="D6" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F6" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H6" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I6" t="str">
+        <v>23BSFT101</v>
+      </c>
+      <c r="J6" t="str">
+        <v>December - 2026</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L6" t="str">
+        <v>V</v>
+      </c>
+      <c r="M6" t="str">
+        <v>GCBSFT00001</v>
+      </c>
+      <c r="N6" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O6" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P6">
+        <v>1</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>SUB101</v>
+      </c>
+      <c r="R6" t="str">
+        <v>Introduction to Subject One</v>
+      </c>
+      <c r="S6">
+        <v>4</v>
+      </c>
+      <c r="T6">
+        <v>4</v>
+      </c>
+      <c r="U6">
+        <v>40</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>16</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <v>30</v>
+      </c>
+      <c r="Z6">
+        <v>0</v>
+      </c>
+      <c r="AA6">
+        <v>60</v>
+      </c>
+      <c r="AB6">
+        <v>0</v>
+      </c>
+      <c r="AC6">
+        <v>24</v>
+      </c>
+      <c r="AD6">
+        <v>0</v>
+      </c>
+      <c r="AE6">
+        <v>45</v>
+      </c>
+      <c r="AF6">
+        <v>0</v>
+      </c>
+      <c r="AG6">
+        <v>100</v>
+      </c>
+      <c r="AH6">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ6" t="str">
+        <v>A</v>
+      </c>
+      <c r="AK6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>23bsft101@gcu.edu.in</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Abigail Albert Anbudurai</v>
+      </c>
+      <c r="D7" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F7" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H7" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I7" t="str">
+        <v>23BSFT101</v>
+      </c>
+      <c r="J7" t="str">
+        <v>December - 2026</v>
+      </c>
+      <c r="K7" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L7" t="str">
+        <v>V</v>
+      </c>
+      <c r="M7" t="str">
+        <v>GCBSFT00001</v>
+      </c>
+      <c r="N7" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O7" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P7">
+        <v>1</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>SUB102</v>
+      </c>
+      <c r="R7" t="str">
+        <v>Introduction to Subject Two</v>
+      </c>
+      <c r="S7">
+        <v>4</v>
+      </c>
+      <c r="T7">
+        <v>4</v>
+      </c>
+      <c r="U7">
+        <v>40</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>16</v>
+      </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7">
+        <v>35.2</v>
+      </c>
+      <c r="Z7">
+        <v>0</v>
+      </c>
+      <c r="AA7">
+        <v>60</v>
+      </c>
+      <c r="AB7">
+        <v>0</v>
+      </c>
+      <c r="AC7">
+        <v>24</v>
+      </c>
+      <c r="AD7">
+        <v>0</v>
+      </c>
+      <c r="AE7">
+        <v>52.8</v>
+      </c>
+      <c r="AF7">
+        <v>0</v>
+      </c>
+      <c r="AG7">
+        <v>100</v>
+      </c>
+      <c r="AH7">
+        <v>0</v>
+      </c>
+      <c r="AI7" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ7" t="str">
+        <v>A+</v>
+      </c>
+      <c r="AK7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>23bsft101@gcu.edu.in</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Abigail Albert Anbudurai</v>
+      </c>
+      <c r="D8" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F8" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H8" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I8" t="str">
+        <v>23BSFT101</v>
+      </c>
+      <c r="J8" t="str">
+        <v>December - 2026</v>
+      </c>
+      <c r="K8" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L8" t="str">
+        <v>V</v>
+      </c>
+      <c r="M8" t="str">
+        <v>GCBSFT00001</v>
+      </c>
+      <c r="N8" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O8" t="str">
+        <v>PRACTICAL</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>SUB103P</v>
+      </c>
+      <c r="R8" t="str">
+        <v>Practical Lab One</v>
+      </c>
+      <c r="S8">
+        <v>4</v>
+      </c>
+      <c r="T8">
+        <v>4</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>40</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <v>16</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
+      <c r="Z8">
+        <v>38</v>
+      </c>
+      <c r="AA8">
+        <v>0</v>
+      </c>
+      <c r="AB8">
+        <v>60</v>
+      </c>
+      <c r="AC8">
+        <v>0</v>
+      </c>
+      <c r="AD8">
+        <v>24</v>
+      </c>
+      <c r="AE8">
+        <v>0</v>
+      </c>
+      <c r="AF8">
+        <v>57</v>
+      </c>
+      <c r="AG8">
+        <v>100</v>
+      </c>
+      <c r="AH8">
+        <v>0</v>
+      </c>
+      <c r="AI8" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ8" t="str">
+        <v>O</v>
+      </c>
+      <c r="AK8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>23bsft101@gcu.edu.in</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Abigail Albert Anbudurai</v>
+      </c>
+      <c r="D9" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F9" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H9" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I9" t="str">
+        <v>23BSFT101</v>
+      </c>
+      <c r="J9" t="str">
+        <v>December - 2026</v>
+      </c>
+      <c r="K9" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L9" t="str">
+        <v>V</v>
+      </c>
+      <c r="M9" t="str">
+        <v>GCBSFT00001</v>
+      </c>
+      <c r="N9" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O9" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P9">
+        <v>1</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>SUB104</v>
+      </c>
+      <c r="R9" t="str">
+        <v>Advanced Subject Four</v>
+      </c>
+      <c r="S9">
+        <v>4</v>
+      </c>
+      <c r="T9">
+        <v>4</v>
+      </c>
+      <c r="U9">
+        <v>40</v>
+      </c>
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
+        <v>16</v>
+      </c>
+      <c r="X9">
+        <v>0</v>
+      </c>
+      <c r="Y9">
+        <v>27.200000000000003</v>
+      </c>
+      <c r="Z9">
+        <v>0</v>
+      </c>
+      <c r="AA9">
+        <v>60</v>
+      </c>
+      <c r="AB9">
+        <v>0</v>
+      </c>
+      <c r="AC9">
+        <v>24</v>
+      </c>
+      <c r="AD9">
+        <v>0</v>
+      </c>
+      <c r="AE9">
+        <v>40.8</v>
+      </c>
+      <c r="AF9">
+        <v>0</v>
+      </c>
+      <c r="AG9">
+        <v>100</v>
+      </c>
+      <c r="AH9">
+        <v>0</v>
+      </c>
+      <c r="AI9" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ9" t="str">
+        <v>B+</v>
+      </c>
+      <c r="AK9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>23bsft102@gcu.edu.in</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Rahul Krishnan</v>
+      </c>
+      <c r="D10" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F10" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H10" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I10" t="str">
+        <v>23BSFT102</v>
+      </c>
+      <c r="J10" t="str">
+        <v>April - 2026</v>
+      </c>
+      <c r="K10" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L10" t="str">
+        <v>IV</v>
+      </c>
+      <c r="M10" t="str">
+        <v>GCBSFT00002</v>
+      </c>
+      <c r="N10" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O10" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P10">
+        <v>1</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>SUB101</v>
+      </c>
+      <c r="R10" t="str">
+        <v>Introduction to Subject One</v>
+      </c>
+      <c r="S10">
+        <v>4</v>
+      </c>
+      <c r="T10">
+        <v>4</v>
+      </c>
+      <c r="U10">
+        <v>40</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>16</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
+        <v>30</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>60</v>
+      </c>
+      <c r="AB10">
+        <v>0</v>
+      </c>
+      <c r="AC10">
+        <v>24</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+      <c r="AE10">
+        <v>45</v>
+      </c>
+      <c r="AF10">
+        <v>0</v>
+      </c>
+      <c r="AG10">
+        <v>100</v>
+      </c>
+      <c r="AH10">
+        <v>0</v>
+      </c>
+      <c r="AI10" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ10" t="str">
+        <v>A</v>
+      </c>
+      <c r="AK10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>23bsft102@gcu.edu.in</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Rahul Krishnan</v>
+      </c>
+      <c r="D11" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F11" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H11" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I11" t="str">
+        <v>23BSFT102</v>
+      </c>
+      <c r="J11" t="str">
+        <v>April - 2026</v>
+      </c>
+      <c r="K11" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L11" t="str">
+        <v>IV</v>
+      </c>
+      <c r="M11" t="str">
+        <v>GCBSFT00002</v>
+      </c>
+      <c r="N11" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O11" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P11">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>SUB102</v>
+      </c>
+      <c r="R11" t="str">
+        <v>Introduction to Subject Two</v>
+      </c>
+      <c r="S11">
+        <v>4</v>
+      </c>
+      <c r="T11">
+        <v>4</v>
+      </c>
+      <c r="U11">
+        <v>40</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>16</v>
+      </c>
+      <c r="X11">
+        <v>0</v>
+      </c>
+      <c r="Y11">
+        <v>35.2</v>
+      </c>
+      <c r="Z11">
+        <v>0</v>
+      </c>
+      <c r="AA11">
+        <v>60</v>
+      </c>
+      <c r="AB11">
+        <v>0</v>
+      </c>
+      <c r="AC11">
+        <v>24</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+      <c r="AE11">
+        <v>52.8</v>
+      </c>
+      <c r="AF11">
+        <v>0</v>
+      </c>
+      <c r="AG11">
+        <v>100</v>
+      </c>
+      <c r="AH11">
+        <v>0</v>
+      </c>
+      <c r="AI11" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ11" t="str">
+        <v>A+</v>
+      </c>
+      <c r="AK11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>23bsft102@gcu.edu.in</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Rahul Krishnan</v>
+      </c>
+      <c r="D12" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F12" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H12" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I12" t="str">
+        <v>23BSFT102</v>
+      </c>
+      <c r="J12" t="str">
+        <v>April - 2026</v>
+      </c>
+      <c r="K12" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L12" t="str">
+        <v>IV</v>
+      </c>
+      <c r="M12" t="str">
+        <v>GCBSFT00002</v>
+      </c>
+      <c r="N12" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O12" t="str">
+        <v>PRACTICAL</v>
+      </c>
+      <c r="P12">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>SUB103P</v>
+      </c>
+      <c r="R12" t="str">
+        <v>Practical Lab One</v>
+      </c>
+      <c r="S12">
+        <v>4</v>
+      </c>
+      <c r="T12">
+        <v>4</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <v>40</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <v>16</v>
+      </c>
+      <c r="Y12">
+        <v>0</v>
+      </c>
+      <c r="Z12">
+        <v>38</v>
+      </c>
+      <c r="AA12">
+        <v>0</v>
+      </c>
+      <c r="AB12">
+        <v>60</v>
+      </c>
+      <c r="AC12">
+        <v>0</v>
+      </c>
+      <c r="AD12">
+        <v>24</v>
+      </c>
+      <c r="AE12">
+        <v>0</v>
+      </c>
+      <c r="AF12">
+        <v>57</v>
+      </c>
+      <c r="AG12">
+        <v>100</v>
+      </c>
+      <c r="AH12">
+        <v>0</v>
+      </c>
+      <c r="AI12" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ12" t="str">
+        <v>O</v>
+      </c>
+      <c r="AK12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>23bsft102@gcu.edu.in</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Rahul Krishnan</v>
+      </c>
+      <c r="D13" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F13" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H13" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I13" t="str">
+        <v>23BSFT102</v>
+      </c>
+      <c r="J13" t="str">
+        <v>April - 2026</v>
+      </c>
+      <c r="K13" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L13" t="str">
+        <v>IV</v>
+      </c>
+      <c r="M13" t="str">
+        <v>GCBSFT00002</v>
+      </c>
+      <c r="N13" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O13" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P13">
+        <v>1</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>SUB104</v>
+      </c>
+      <c r="R13" t="str">
+        <v>Advanced Subject Four</v>
+      </c>
+      <c r="S13">
+        <v>4</v>
+      </c>
+      <c r="T13">
+        <v>4</v>
+      </c>
+      <c r="U13">
+        <v>40</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>16</v>
+      </c>
+      <c r="X13">
+        <v>0</v>
+      </c>
+      <c r="Y13">
+        <v>27.200000000000003</v>
+      </c>
+      <c r="Z13">
+        <v>0</v>
+      </c>
+      <c r="AA13">
+        <v>60</v>
+      </c>
+      <c r="AB13">
+        <v>0</v>
+      </c>
+      <c r="AC13">
+        <v>24</v>
+      </c>
+      <c r="AD13">
+        <v>0</v>
+      </c>
+      <c r="AE13">
+        <v>40.8</v>
+      </c>
+      <c r="AF13">
+        <v>0</v>
+      </c>
+      <c r="AG13">
+        <v>100</v>
+      </c>
+      <c r="AH13">
+        <v>0</v>
+      </c>
+      <c r="AI13" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ13" t="str">
+        <v>B+</v>
+      </c>
+      <c r="AK13">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>23bsft102@gcu.edu.in</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Rahul Krishnan</v>
+      </c>
+      <c r="D14" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F14" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H14" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I14" t="str">
+        <v>23BSFT102</v>
+      </c>
+      <c r="J14" t="str">
+        <v>December - 2026</v>
+      </c>
+      <c r="K14" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L14" t="str">
+        <v>V</v>
+      </c>
+      <c r="M14" t="str">
+        <v>GCBSFT00002</v>
+      </c>
+      <c r="N14" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O14" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P14">
+        <v>1</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>SUB101</v>
+      </c>
+      <c r="R14" t="str">
+        <v>Introduction to Subject One</v>
+      </c>
+      <c r="S14">
+        <v>4</v>
+      </c>
+      <c r="T14">
+        <v>4</v>
+      </c>
+      <c r="U14">
+        <v>40</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>16</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
+      <c r="Y14">
+        <v>30</v>
+      </c>
+      <c r="Z14">
+        <v>0</v>
+      </c>
+      <c r="AA14">
+        <v>60</v>
+      </c>
+      <c r="AB14">
+        <v>0</v>
+      </c>
+      <c r="AC14">
+        <v>24</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
+      </c>
+      <c r="AE14">
+        <v>45</v>
+      </c>
+      <c r="AF14">
+        <v>0</v>
+      </c>
+      <c r="AG14">
+        <v>100</v>
+      </c>
+      <c r="AH14">
+        <v>0</v>
+      </c>
+      <c r="AI14" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ14" t="str">
+        <v>A</v>
+      </c>
+      <c r="AK14">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>23bsft102@gcu.edu.in</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Rahul Krishnan</v>
+      </c>
+      <c r="D15" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F15" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H15" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I15" t="str">
+        <v>23BSFT102</v>
+      </c>
+      <c r="J15" t="str">
+        <v>December - 2026</v>
+      </c>
+      <c r="K15" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L15" t="str">
+        <v>V</v>
+      </c>
+      <c r="M15" t="str">
+        <v>GCBSFT00002</v>
+      </c>
+      <c r="N15" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O15" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P15">
+        <v>1</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>SUB102</v>
+      </c>
+      <c r="R15" t="str">
+        <v>Introduction to Subject Two</v>
+      </c>
+      <c r="S15">
+        <v>4</v>
+      </c>
+      <c r="T15">
+        <v>4</v>
+      </c>
+      <c r="U15">
+        <v>40</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <v>16</v>
+      </c>
+      <c r="X15">
+        <v>0</v>
+      </c>
+      <c r="Y15">
+        <v>35.2</v>
+      </c>
+      <c r="Z15">
+        <v>0</v>
+      </c>
+      <c r="AA15">
+        <v>60</v>
+      </c>
+      <c r="AB15">
+        <v>0</v>
+      </c>
+      <c r="AC15">
+        <v>24</v>
+      </c>
+      <c r="AD15">
+        <v>0</v>
+      </c>
+      <c r="AE15">
+        <v>52.8</v>
+      </c>
+      <c r="AF15">
+        <v>0</v>
+      </c>
+      <c r="AG15">
+        <v>100</v>
+      </c>
+      <c r="AH15">
+        <v>0</v>
+      </c>
+      <c r="AI15" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ15" t="str">
+        <v>A+</v>
+      </c>
+      <c r="AK15">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>23bsft102@gcu.edu.in</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Rahul Krishnan</v>
+      </c>
+      <c r="D16" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F16" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H16" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I16" t="str">
+        <v>23BSFT102</v>
+      </c>
+      <c r="J16" t="str">
+        <v>December - 2026</v>
+      </c>
+      <c r="K16" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L16" t="str">
+        <v>V</v>
+      </c>
+      <c r="M16" t="str">
+        <v>GCBSFT00002</v>
+      </c>
+      <c r="N16" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O16" t="str">
+        <v>PRACTICAL</v>
+      </c>
+      <c r="P16">
+        <v>1</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>SUB103P</v>
+      </c>
+      <c r="R16" t="str">
+        <v>Practical Lab One</v>
+      </c>
+      <c r="S16">
+        <v>4</v>
+      </c>
+      <c r="T16">
+        <v>4</v>
+      </c>
+      <c r="U16">
+        <v>0</v>
+      </c>
+      <c r="V16">
+        <v>40</v>
+      </c>
+      <c r="W16">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>16</v>
+      </c>
+      <c r="Y16">
+        <v>0</v>
+      </c>
+      <c r="Z16">
+        <v>38</v>
+      </c>
+      <c r="AA16">
+        <v>0</v>
+      </c>
+      <c r="AB16">
+        <v>60</v>
+      </c>
+      <c r="AC16">
+        <v>0</v>
+      </c>
+      <c r="AD16">
+        <v>24</v>
+      </c>
+      <c r="AE16">
+        <v>0</v>
+      </c>
+      <c r="AF16">
+        <v>57</v>
+      </c>
+      <c r="AG16">
+        <v>100</v>
+      </c>
+      <c r="AH16">
+        <v>0</v>
+      </c>
+      <c r="AI16" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ16" t="str">
+        <v>O</v>
+      </c>
+      <c r="AK16">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>23bsft102@gcu.edu.in</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Rahul Krishnan</v>
+      </c>
+      <c r="D17" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Garden City University</v>
+      </c>
+      <c r="F17" t="str">
+        <v>SCHOOL OF SCIENCES</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Bachelor of Science Food Science and Technology</v>
+      </c>
+      <c r="H17" t="str">
+        <v>BSFT</v>
+      </c>
+      <c r="I17" t="str">
+        <v>23BSFT102</v>
+      </c>
+      <c r="J17" t="str">
+        <v>December - 2026</v>
+      </c>
+      <c r="K17" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="L17" t="str">
+        <v>V</v>
+      </c>
+      <c r="M17" t="str">
+        <v>GCBSFT00002</v>
+      </c>
+      <c r="N17" t="str">
+        <v>CORE COURSE</v>
+      </c>
+      <c r="O17" t="str">
+        <v>THEORY</v>
+      </c>
+      <c r="P17">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>SUB104</v>
+      </c>
+      <c r="R17" t="str">
+        <v>Advanced Subject Four</v>
+      </c>
+      <c r="S17">
+        <v>4</v>
+      </c>
+      <c r="T17">
+        <v>4</v>
+      </c>
+      <c r="U17">
+        <v>40</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+      <c r="W17">
+        <v>16</v>
+      </c>
+      <c r="X17">
+        <v>0</v>
+      </c>
+      <c r="Y17">
+        <v>27.200000000000003</v>
+      </c>
+      <c r="Z17">
+        <v>0</v>
+      </c>
+      <c r="AA17">
+        <v>60</v>
+      </c>
+      <c r="AB17">
+        <v>0</v>
+      </c>
+      <c r="AC17">
+        <v>24</v>
+      </c>
+      <c r="AD17">
+        <v>0</v>
+      </c>
+      <c r="AE17">
+        <v>40.8</v>
+      </c>
+      <c r="AF17">
+        <v>0</v>
+      </c>
+      <c r="AG17">
+        <v>100</v>
+      </c>
+      <c r="AH17">
+        <v>0</v>
+      </c>
+      <c r="AI17" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="AJ17" t="str">
+        <v>B+</v>
+      </c>
+      <c r="AK17">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AL2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AK17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add marks configuration, simplified Excel upload, and COE portal renames.
Introduce configurable CIA/ESE limits, unified obtained-marks columns, per-student photo resolution, and migrate super-admin/faculty routes to COE/admin with supporting Supabase migrations.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/marks_template_final.xlsx
+++ b/public/marks_template_final.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK17"/>
+  <dimension ref="A1:Y17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -461,54 +461,18 @@
         <v>Credits Earned</v>
       </c>
       <c r="U1" t="str">
-        <v>CIA Max Marks Theory</v>
+        <v>CIA Marks Obtained</v>
       </c>
       <c r="V1" t="str">
-        <v>CIA Max Marks Practical</v>
+        <v>ESE Marks Obtained</v>
       </c>
       <c r="W1" t="str">
-        <v>CIA Min Marks Theory</v>
+        <v>Status</v>
       </c>
       <c r="X1" t="str">
-        <v>CIA Min Marks Practical</v>
+        <v>Grade Obtained</v>
       </c>
       <c r="Y1" t="str">
-        <v>CIA Marks Obtained Theory</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>CIA Marks Obtained Practical</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>ESE Max Marks Theory</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>ESE Max Marks Practical</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>ESE Min Marks Theory</v>
-      </c>
-      <c r="AD1" t="str">
-        <v>ESE Min Marks Practical</v>
-      </c>
-      <c r="AE1" t="str">
-        <v>ESE Marks Obtained Theory</v>
-      </c>
-      <c r="AF1" t="str">
-        <v>ESE Marks Obtained Practical</v>
-      </c>
-      <c r="AG1" t="str">
-        <v>Total Marks Theory</v>
-      </c>
-      <c r="AH1" t="str">
-        <v>Total Marks Practical</v>
-      </c>
-      <c r="AI1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="AJ1" t="str">
-        <v>Grade Obtained</v>
-      </c>
-      <c r="AK1" t="str">
         <v>Grade Points</v>
       </c>
     </row>
@@ -574,54 +538,18 @@
         <v>4</v>
       </c>
       <c r="U2">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="V2">
-        <v>0</v>
-      </c>
-      <c r="W2">
-        <v>16</v>
-      </c>
-      <c r="X2">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="W2" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X2" t="str">
+        <v>A</v>
       </c>
       <c r="Y2">
-        <v>30</v>
-      </c>
-      <c r="Z2">
-        <v>0</v>
-      </c>
-      <c r="AA2">
-        <v>60</v>
-      </c>
-      <c r="AB2">
-        <v>0</v>
-      </c>
-      <c r="AC2">
-        <v>24</v>
-      </c>
-      <c r="AD2">
-        <v>0</v>
-      </c>
-      <c r="AE2">
-        <v>45</v>
-      </c>
-      <c r="AF2">
-        <v>0</v>
-      </c>
-      <c r="AG2">
-        <v>100</v>
-      </c>
-      <c r="AH2">
-        <v>0</v>
-      </c>
-      <c r="AI2" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ2" t="str">
-        <v>A</v>
-      </c>
-      <c r="AK2">
         <v>8</v>
       </c>
     </row>
@@ -687,54 +615,18 @@
         <v>4</v>
       </c>
       <c r="U3">
-        <v>40</v>
+        <v>35.2</v>
       </c>
       <c r="V3">
-        <v>0</v>
-      </c>
-      <c r="W3">
-        <v>16</v>
-      </c>
-      <c r="X3">
-        <v>0</v>
+        <v>52.8</v>
+      </c>
+      <c r="W3" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X3" t="str">
+        <v>A+</v>
       </c>
       <c r="Y3">
-        <v>35.2</v>
-      </c>
-      <c r="Z3">
-        <v>0</v>
-      </c>
-      <c r="AA3">
-        <v>60</v>
-      </c>
-      <c r="AB3">
-        <v>0</v>
-      </c>
-      <c r="AC3">
-        <v>24</v>
-      </c>
-      <c r="AD3">
-        <v>0</v>
-      </c>
-      <c r="AE3">
-        <v>52.8</v>
-      </c>
-      <c r="AF3">
-        <v>0</v>
-      </c>
-      <c r="AG3">
-        <v>100</v>
-      </c>
-      <c r="AH3">
-        <v>0</v>
-      </c>
-      <c r="AI3" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ3" t="str">
-        <v>A+</v>
-      </c>
-      <c r="AK3">
         <v>9</v>
       </c>
     </row>
@@ -800,54 +692,18 @@
         <v>4</v>
       </c>
       <c r="U4">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="V4">
-        <v>40</v>
-      </c>
-      <c r="W4">
-        <v>0</v>
-      </c>
-      <c r="X4">
-        <v>16</v>
+        <v>57</v>
+      </c>
+      <c r="W4" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X4" t="str">
+        <v>O</v>
       </c>
       <c r="Y4">
-        <v>0</v>
-      </c>
-      <c r="Z4">
-        <v>38</v>
-      </c>
-      <c r="AA4">
-        <v>0</v>
-      </c>
-      <c r="AB4">
-        <v>60</v>
-      </c>
-      <c r="AC4">
-        <v>0</v>
-      </c>
-      <c r="AD4">
-        <v>24</v>
-      </c>
-      <c r="AE4">
-        <v>0</v>
-      </c>
-      <c r="AF4">
-        <v>57</v>
-      </c>
-      <c r="AG4">
-        <v>100</v>
-      </c>
-      <c r="AH4">
-        <v>0</v>
-      </c>
-      <c r="AI4" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ4" t="str">
-        <v>O</v>
-      </c>
-      <c r="AK4">
         <v>10</v>
       </c>
     </row>
@@ -913,54 +769,18 @@
         <v>4</v>
       </c>
       <c r="U5">
-        <v>40</v>
+        <v>27.200000000000003</v>
       </c>
       <c r="V5">
-        <v>0</v>
-      </c>
-      <c r="W5">
-        <v>16</v>
-      </c>
-      <c r="X5">
-        <v>0</v>
+        <v>40.8</v>
+      </c>
+      <c r="W5" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X5" t="str">
+        <v>B+</v>
       </c>
       <c r="Y5">
-        <v>27.200000000000003</v>
-      </c>
-      <c r="Z5">
-        <v>0</v>
-      </c>
-      <c r="AA5">
-        <v>60</v>
-      </c>
-      <c r="AB5">
-        <v>0</v>
-      </c>
-      <c r="AC5">
-        <v>24</v>
-      </c>
-      <c r="AD5">
-        <v>0</v>
-      </c>
-      <c r="AE5">
-        <v>40.8</v>
-      </c>
-      <c r="AF5">
-        <v>0</v>
-      </c>
-      <c r="AG5">
-        <v>100</v>
-      </c>
-      <c r="AH5">
-        <v>0</v>
-      </c>
-      <c r="AI5" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ5" t="str">
-        <v>B+</v>
-      </c>
-      <c r="AK5">
         <v>7</v>
       </c>
     </row>
@@ -1026,54 +846,18 @@
         <v>4</v>
       </c>
       <c r="U6">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="V6">
-        <v>0</v>
-      </c>
-      <c r="W6">
-        <v>16</v>
-      </c>
-      <c r="X6">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="W6" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X6" t="str">
+        <v>A</v>
       </c>
       <c r="Y6">
-        <v>30</v>
-      </c>
-      <c r="Z6">
-        <v>0</v>
-      </c>
-      <c r="AA6">
-        <v>60</v>
-      </c>
-      <c r="AB6">
-        <v>0</v>
-      </c>
-      <c r="AC6">
-        <v>24</v>
-      </c>
-      <c r="AD6">
-        <v>0</v>
-      </c>
-      <c r="AE6">
-        <v>45</v>
-      </c>
-      <c r="AF6">
-        <v>0</v>
-      </c>
-      <c r="AG6">
-        <v>100</v>
-      </c>
-      <c r="AH6">
-        <v>0</v>
-      </c>
-      <c r="AI6" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ6" t="str">
-        <v>A</v>
-      </c>
-      <c r="AK6">
         <v>8</v>
       </c>
     </row>
@@ -1139,54 +923,18 @@
         <v>4</v>
       </c>
       <c r="U7">
-        <v>40</v>
+        <v>35.2</v>
       </c>
       <c r="V7">
-        <v>0</v>
-      </c>
-      <c r="W7">
-        <v>16</v>
-      </c>
-      <c r="X7">
-        <v>0</v>
+        <v>52.8</v>
+      </c>
+      <c r="W7" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X7" t="str">
+        <v>A+</v>
       </c>
       <c r="Y7">
-        <v>35.2</v>
-      </c>
-      <c r="Z7">
-        <v>0</v>
-      </c>
-      <c r="AA7">
-        <v>60</v>
-      </c>
-      <c r="AB7">
-        <v>0</v>
-      </c>
-      <c r="AC7">
-        <v>24</v>
-      </c>
-      <c r="AD7">
-        <v>0</v>
-      </c>
-      <c r="AE7">
-        <v>52.8</v>
-      </c>
-      <c r="AF7">
-        <v>0</v>
-      </c>
-      <c r="AG7">
-        <v>100</v>
-      </c>
-      <c r="AH7">
-        <v>0</v>
-      </c>
-      <c r="AI7" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ7" t="str">
-        <v>A+</v>
-      </c>
-      <c r="AK7">
         <v>9</v>
       </c>
     </row>
@@ -1252,54 +1000,18 @@
         <v>4</v>
       </c>
       <c r="U8">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="V8">
-        <v>40</v>
-      </c>
-      <c r="W8">
-        <v>0</v>
-      </c>
-      <c r="X8">
-        <v>16</v>
+        <v>57</v>
+      </c>
+      <c r="W8" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X8" t="str">
+        <v>O</v>
       </c>
       <c r="Y8">
-        <v>0</v>
-      </c>
-      <c r="Z8">
-        <v>38</v>
-      </c>
-      <c r="AA8">
-        <v>0</v>
-      </c>
-      <c r="AB8">
-        <v>60</v>
-      </c>
-      <c r="AC8">
-        <v>0</v>
-      </c>
-      <c r="AD8">
-        <v>24</v>
-      </c>
-      <c r="AE8">
-        <v>0</v>
-      </c>
-      <c r="AF8">
-        <v>57</v>
-      </c>
-      <c r="AG8">
-        <v>100</v>
-      </c>
-      <c r="AH8">
-        <v>0</v>
-      </c>
-      <c r="AI8" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ8" t="str">
-        <v>O</v>
-      </c>
-      <c r="AK8">
         <v>10</v>
       </c>
     </row>
@@ -1365,54 +1077,18 @@
         <v>4</v>
       </c>
       <c r="U9">
-        <v>40</v>
+        <v>27.200000000000003</v>
       </c>
       <c r="V9">
-        <v>0</v>
-      </c>
-      <c r="W9">
-        <v>16</v>
-      </c>
-      <c r="X9">
-        <v>0</v>
+        <v>40.8</v>
+      </c>
+      <c r="W9" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X9" t="str">
+        <v>B+</v>
       </c>
       <c r="Y9">
-        <v>27.200000000000003</v>
-      </c>
-      <c r="Z9">
-        <v>0</v>
-      </c>
-      <c r="AA9">
-        <v>60</v>
-      </c>
-      <c r="AB9">
-        <v>0</v>
-      </c>
-      <c r="AC9">
-        <v>24</v>
-      </c>
-      <c r="AD9">
-        <v>0</v>
-      </c>
-      <c r="AE9">
-        <v>40.8</v>
-      </c>
-      <c r="AF9">
-        <v>0</v>
-      </c>
-      <c r="AG9">
-        <v>100</v>
-      </c>
-      <c r="AH9">
-        <v>0</v>
-      </c>
-      <c r="AI9" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ9" t="str">
-        <v>B+</v>
-      </c>
-      <c r="AK9">
         <v>7</v>
       </c>
     </row>
@@ -1478,54 +1154,18 @@
         <v>4</v>
       </c>
       <c r="U10">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="V10">
-        <v>0</v>
-      </c>
-      <c r="W10">
-        <v>16</v>
-      </c>
-      <c r="X10">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="W10" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X10" t="str">
+        <v>A</v>
       </c>
       <c r="Y10">
-        <v>30</v>
-      </c>
-      <c r="Z10">
-        <v>0</v>
-      </c>
-      <c r="AA10">
-        <v>60</v>
-      </c>
-      <c r="AB10">
-        <v>0</v>
-      </c>
-      <c r="AC10">
-        <v>24</v>
-      </c>
-      <c r="AD10">
-        <v>0</v>
-      </c>
-      <c r="AE10">
-        <v>45</v>
-      </c>
-      <c r="AF10">
-        <v>0</v>
-      </c>
-      <c r="AG10">
-        <v>100</v>
-      </c>
-      <c r="AH10">
-        <v>0</v>
-      </c>
-      <c r="AI10" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ10" t="str">
-        <v>A</v>
-      </c>
-      <c r="AK10">
         <v>8</v>
       </c>
     </row>
@@ -1591,54 +1231,18 @@
         <v>4</v>
       </c>
       <c r="U11">
-        <v>40</v>
+        <v>35.2</v>
       </c>
       <c r="V11">
-        <v>0</v>
-      </c>
-      <c r="W11">
-        <v>16</v>
-      </c>
-      <c r="X11">
-        <v>0</v>
+        <v>52.8</v>
+      </c>
+      <c r="W11" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X11" t="str">
+        <v>A+</v>
       </c>
       <c r="Y11">
-        <v>35.2</v>
-      </c>
-      <c r="Z11">
-        <v>0</v>
-      </c>
-      <c r="AA11">
-        <v>60</v>
-      </c>
-      <c r="AB11">
-        <v>0</v>
-      </c>
-      <c r="AC11">
-        <v>24</v>
-      </c>
-      <c r="AD11">
-        <v>0</v>
-      </c>
-      <c r="AE11">
-        <v>52.8</v>
-      </c>
-      <c r="AF11">
-        <v>0</v>
-      </c>
-      <c r="AG11">
-        <v>100</v>
-      </c>
-      <c r="AH11">
-        <v>0</v>
-      </c>
-      <c r="AI11" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ11" t="str">
-        <v>A+</v>
-      </c>
-      <c r="AK11">
         <v>9</v>
       </c>
     </row>
@@ -1704,54 +1308,18 @@
         <v>4</v>
       </c>
       <c r="U12">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="V12">
-        <v>40</v>
-      </c>
-      <c r="W12">
-        <v>0</v>
-      </c>
-      <c r="X12">
-        <v>16</v>
+        <v>57</v>
+      </c>
+      <c r="W12" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X12" t="str">
+        <v>O</v>
       </c>
       <c r="Y12">
-        <v>0</v>
-      </c>
-      <c r="Z12">
-        <v>38</v>
-      </c>
-      <c r="AA12">
-        <v>0</v>
-      </c>
-      <c r="AB12">
-        <v>60</v>
-      </c>
-      <c r="AC12">
-        <v>0</v>
-      </c>
-      <c r="AD12">
-        <v>24</v>
-      </c>
-      <c r="AE12">
-        <v>0</v>
-      </c>
-      <c r="AF12">
-        <v>57</v>
-      </c>
-      <c r="AG12">
-        <v>100</v>
-      </c>
-      <c r="AH12">
-        <v>0</v>
-      </c>
-      <c r="AI12" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ12" t="str">
-        <v>O</v>
-      </c>
-      <c r="AK12">
         <v>10</v>
       </c>
     </row>
@@ -1817,54 +1385,18 @@
         <v>4</v>
       </c>
       <c r="U13">
-        <v>40</v>
+        <v>27.200000000000003</v>
       </c>
       <c r="V13">
-        <v>0</v>
-      </c>
-      <c r="W13">
-        <v>16</v>
-      </c>
-      <c r="X13">
-        <v>0</v>
+        <v>40.8</v>
+      </c>
+      <c r="W13" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X13" t="str">
+        <v>B+</v>
       </c>
       <c r="Y13">
-        <v>27.200000000000003</v>
-      </c>
-      <c r="Z13">
-        <v>0</v>
-      </c>
-      <c r="AA13">
-        <v>60</v>
-      </c>
-      <c r="AB13">
-        <v>0</v>
-      </c>
-      <c r="AC13">
-        <v>24</v>
-      </c>
-      <c r="AD13">
-        <v>0</v>
-      </c>
-      <c r="AE13">
-        <v>40.8</v>
-      </c>
-      <c r="AF13">
-        <v>0</v>
-      </c>
-      <c r="AG13">
-        <v>100</v>
-      </c>
-      <c r="AH13">
-        <v>0</v>
-      </c>
-      <c r="AI13" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ13" t="str">
-        <v>B+</v>
-      </c>
-      <c r="AK13">
         <v>7</v>
       </c>
     </row>
@@ -1930,54 +1462,18 @@
         <v>4</v>
       </c>
       <c r="U14">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="V14">
-        <v>0</v>
-      </c>
-      <c r="W14">
-        <v>16</v>
-      </c>
-      <c r="X14">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="W14" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X14" t="str">
+        <v>A</v>
       </c>
       <c r="Y14">
-        <v>30</v>
-      </c>
-      <c r="Z14">
-        <v>0</v>
-      </c>
-      <c r="AA14">
-        <v>60</v>
-      </c>
-      <c r="AB14">
-        <v>0</v>
-      </c>
-      <c r="AC14">
-        <v>24</v>
-      </c>
-      <c r="AD14">
-        <v>0</v>
-      </c>
-      <c r="AE14">
-        <v>45</v>
-      </c>
-      <c r="AF14">
-        <v>0</v>
-      </c>
-      <c r="AG14">
-        <v>100</v>
-      </c>
-      <c r="AH14">
-        <v>0</v>
-      </c>
-      <c r="AI14" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ14" t="str">
-        <v>A</v>
-      </c>
-      <c r="AK14">
         <v>8</v>
       </c>
     </row>
@@ -2043,54 +1539,18 @@
         <v>4</v>
       </c>
       <c r="U15">
-        <v>40</v>
+        <v>35.2</v>
       </c>
       <c r="V15">
-        <v>0</v>
-      </c>
-      <c r="W15">
-        <v>16</v>
-      </c>
-      <c r="X15">
-        <v>0</v>
+        <v>52.8</v>
+      </c>
+      <c r="W15" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X15" t="str">
+        <v>A+</v>
       </c>
       <c r="Y15">
-        <v>35.2</v>
-      </c>
-      <c r="Z15">
-        <v>0</v>
-      </c>
-      <c r="AA15">
-        <v>60</v>
-      </c>
-      <c r="AB15">
-        <v>0</v>
-      </c>
-      <c r="AC15">
-        <v>24</v>
-      </c>
-      <c r="AD15">
-        <v>0</v>
-      </c>
-      <c r="AE15">
-        <v>52.8</v>
-      </c>
-      <c r="AF15">
-        <v>0</v>
-      </c>
-      <c r="AG15">
-        <v>100</v>
-      </c>
-      <c r="AH15">
-        <v>0</v>
-      </c>
-      <c r="AI15" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ15" t="str">
-        <v>A+</v>
-      </c>
-      <c r="AK15">
         <v>9</v>
       </c>
     </row>
@@ -2156,54 +1616,18 @@
         <v>4</v>
       </c>
       <c r="U16">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="V16">
-        <v>40</v>
-      </c>
-      <c r="W16">
-        <v>0</v>
-      </c>
-      <c r="X16">
-        <v>16</v>
+        <v>57</v>
+      </c>
+      <c r="W16" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X16" t="str">
+        <v>O</v>
       </c>
       <c r="Y16">
-        <v>0</v>
-      </c>
-      <c r="Z16">
-        <v>38</v>
-      </c>
-      <c r="AA16">
-        <v>0</v>
-      </c>
-      <c r="AB16">
-        <v>60</v>
-      </c>
-      <c r="AC16">
-        <v>0</v>
-      </c>
-      <c r="AD16">
-        <v>24</v>
-      </c>
-      <c r="AE16">
-        <v>0</v>
-      </c>
-      <c r="AF16">
-        <v>57</v>
-      </c>
-      <c r="AG16">
-        <v>100</v>
-      </c>
-      <c r="AH16">
-        <v>0</v>
-      </c>
-      <c r="AI16" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ16" t="str">
-        <v>O</v>
-      </c>
-      <c r="AK16">
         <v>10</v>
       </c>
     </row>
@@ -2269,60 +1693,24 @@
         <v>4</v>
       </c>
       <c r="U17">
-        <v>40</v>
+        <v>27.200000000000003</v>
       </c>
       <c r="V17">
-        <v>0</v>
-      </c>
-      <c r="W17">
-        <v>16</v>
-      </c>
-      <c r="X17">
-        <v>0</v>
+        <v>40.8</v>
+      </c>
+      <c r="W17" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="X17" t="str">
+        <v>B+</v>
       </c>
       <c r="Y17">
-        <v>27.200000000000003</v>
-      </c>
-      <c r="Z17">
-        <v>0</v>
-      </c>
-      <c r="AA17">
-        <v>60</v>
-      </c>
-      <c r="AB17">
-        <v>0</v>
-      </c>
-      <c r="AC17">
-        <v>24</v>
-      </c>
-      <c r="AD17">
-        <v>0</v>
-      </c>
-      <c r="AE17">
-        <v>40.8</v>
-      </c>
-      <c r="AF17">
-        <v>0</v>
-      </c>
-      <c r="AG17">
-        <v>100</v>
-      </c>
-      <c r="AH17">
-        <v>0</v>
-      </c>
-      <c r="AI17" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="AJ17" t="str">
-        <v>B+</v>
-      </c>
-      <c r="AK17">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AK17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix marks config, upload compatibility, and legacy portal login routing.
Map admin_2/admin_1 to current roles so staff reach the correct portal after sign-in; add marks configuration storage fallback and relaxed ESE-zero validation when the DB table is missing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/marks_template_final.xlsx
+++ b/public/marks_template_final.xlsx
@@ -461,10 +461,10 @@
         <v>Credits Earned</v>
       </c>
       <c r="U1" t="str">
-        <v>CIA Marks Obtained</v>
+        <v>CIA Obtained</v>
       </c>
       <c r="V1" t="str">
-        <v>ESE Marks Obtained</v>
+        <v>ESE Obtained</v>
       </c>
       <c r="W1" t="str">
         <v>Status</v>

</xml_diff>

<commit_message>
Update COE marks template and tighten controller signature label.
Simplify the sample Excel to one semester with six theory and two practical courses, and position the Controller of Examinations title directly below signature ink in grade and marks card preview and PDF output.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/marks_template_final.xlsx
+++ b/public/marks_template_final.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y17"/>
+  <dimension ref="A1:Y9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -511,7 +511,7 @@
         <v>2026-05-04</v>
       </c>
       <c r="L2" t="str">
-        <v>IV</v>
+        <v>I</v>
       </c>
       <c r="M2" t="str">
         <v>GCBSFT00001</v>
@@ -588,7 +588,7 @@
         <v>2026-05-04</v>
       </c>
       <c r="L3" t="str">
-        <v>IV</v>
+        <v>I</v>
       </c>
       <c r="M3" t="str">
         <v>GCBSFT00001</v>
@@ -665,7 +665,7 @@
         <v>2026-05-04</v>
       </c>
       <c r="L4" t="str">
-        <v>IV</v>
+        <v>I</v>
       </c>
       <c r="M4" t="str">
         <v>GCBSFT00001</v>
@@ -674,16 +674,16 @@
         <v>CORE COURSE</v>
       </c>
       <c r="O4" t="str">
-        <v>PRACTICAL</v>
+        <v>THEORY</v>
       </c>
       <c r="P4">
         <v>1</v>
       </c>
       <c r="Q4" t="str">
-        <v>SUB103P</v>
+        <v>SUB103</v>
       </c>
       <c r="R4" t="str">
-        <v>Practical Lab One</v>
+        <v>Introduction to Subject Three</v>
       </c>
       <c r="S4">
         <v>4</v>
@@ -692,19 +692,19 @@
         <v>4</v>
       </c>
       <c r="U4">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="V4">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="W4" t="str">
         <v>PASS</v>
       </c>
       <c r="X4" t="str">
-        <v>O</v>
+        <v>A</v>
       </c>
       <c r="Y4">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -742,7 +742,7 @@
         <v>2026-05-04</v>
       </c>
       <c r="L5" t="str">
-        <v>IV</v>
+        <v>I</v>
       </c>
       <c r="M5" t="str">
         <v>GCBSFT00001</v>
@@ -813,13 +813,13 @@
         <v>23BSFT101</v>
       </c>
       <c r="J6" t="str">
-        <v>December - 2026</v>
+        <v>April - 2026</v>
       </c>
       <c r="K6" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="L6" t="str">
-        <v>V</v>
+        <v>I</v>
       </c>
       <c r="M6" t="str">
         <v>GCBSFT00001</v>
@@ -834,10 +834,10 @@
         <v>1</v>
       </c>
       <c r="Q6" t="str">
-        <v>SUB101</v>
+        <v>SUB105</v>
       </c>
       <c r="R6" t="str">
-        <v>Introduction to Subject One</v>
+        <v>Introduction to Subject Five</v>
       </c>
       <c r="S6">
         <v>4</v>
@@ -890,13 +890,13 @@
         <v>23BSFT101</v>
       </c>
       <c r="J7" t="str">
-        <v>December - 2026</v>
+        <v>April - 2026</v>
       </c>
       <c r="K7" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="L7" t="str">
-        <v>V</v>
+        <v>I</v>
       </c>
       <c r="M7" t="str">
         <v>GCBSFT00001</v>
@@ -911,10 +911,10 @@
         <v>1</v>
       </c>
       <c r="Q7" t="str">
-        <v>SUB102</v>
+        <v>SUB106</v>
       </c>
       <c r="R7" t="str">
-        <v>Introduction to Subject Two</v>
+        <v>Introduction to Subject Six</v>
       </c>
       <c r="S7">
         <v>4</v>
@@ -967,13 +967,13 @@
         <v>23BSFT101</v>
       </c>
       <c r="J8" t="str">
-        <v>December - 2026</v>
+        <v>April - 2026</v>
       </c>
       <c r="K8" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="L8" t="str">
-        <v>V</v>
+        <v>I</v>
       </c>
       <c r="M8" t="str">
         <v>GCBSFT00001</v>
@@ -988,7 +988,7 @@
         <v>1</v>
       </c>
       <c r="Q8" t="str">
-        <v>SUB103P</v>
+        <v>SUB107P</v>
       </c>
       <c r="R8" t="str">
         <v>Practical Lab One</v>
@@ -1044,13 +1044,13 @@
         <v>23BSFT101</v>
       </c>
       <c r="J9" t="str">
-        <v>December - 2026</v>
+        <v>April - 2026</v>
       </c>
       <c r="K9" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="L9" t="str">
-        <v>V</v>
+        <v>I</v>
       </c>
       <c r="M9" t="str">
         <v>GCBSFT00001</v>
@@ -1059,16 +1059,16 @@
         <v>CORE COURSE</v>
       </c>
       <c r="O9" t="str">
-        <v>THEORY</v>
+        <v>PRACTICAL</v>
       </c>
       <c r="P9">
         <v>1</v>
       </c>
       <c r="Q9" t="str">
-        <v>SUB104</v>
+        <v>SUB108P</v>
       </c>
       <c r="R9" t="str">
-        <v>Advanced Subject Four</v>
+        <v>Practical Lab Two</v>
       </c>
       <c r="S9">
         <v>4</v>
@@ -1077,640 +1077,24 @@
         <v>4</v>
       </c>
       <c r="U9">
-        <v>27.200000000000003</v>
+        <v>38</v>
       </c>
       <c r="V9">
-        <v>40.8</v>
+        <v>57</v>
       </c>
       <c r="W9" t="str">
         <v>PASS</v>
       </c>
       <c r="X9" t="str">
-        <v>B+</v>
+        <v>O</v>
       </c>
       <c r="Y9">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>23bsft102@gcu.edu.in</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Rahul Krishnan</v>
-      </c>
-      <c r="D10" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Garden City University</v>
-      </c>
-      <c r="F10" t="str">
-        <v>SCHOOL OF SCIENCES</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Bachelor of Science Food Science and Technology</v>
-      </c>
-      <c r="H10" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="I10" t="str">
-        <v>23BSFT102</v>
-      </c>
-      <c r="J10" t="str">
-        <v>April - 2026</v>
-      </c>
-      <c r="K10" t="str">
-        <v>2026-05-04</v>
-      </c>
-      <c r="L10" t="str">
-        <v>IV</v>
-      </c>
-      <c r="M10" t="str">
-        <v>GCBSFT00002</v>
-      </c>
-      <c r="N10" t="str">
-        <v>CORE COURSE</v>
-      </c>
-      <c r="O10" t="str">
-        <v>THEORY</v>
-      </c>
-      <c r="P10">
-        <v>1</v>
-      </c>
-      <c r="Q10" t="str">
-        <v>SUB101</v>
-      </c>
-      <c r="R10" t="str">
-        <v>Introduction to Subject One</v>
-      </c>
-      <c r="S10">
-        <v>4</v>
-      </c>
-      <c r="T10">
-        <v>4</v>
-      </c>
-      <c r="U10">
-        <v>30</v>
-      </c>
-      <c r="V10">
-        <v>45</v>
-      </c>
-      <c r="W10" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="X10" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y10">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
         <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>23bsft102@gcu.edu.in</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Rahul Krishnan</v>
-      </c>
-      <c r="D11" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Garden City University</v>
-      </c>
-      <c r="F11" t="str">
-        <v>SCHOOL OF SCIENCES</v>
-      </c>
-      <c r="G11" t="str">
-        <v>Bachelor of Science Food Science and Technology</v>
-      </c>
-      <c r="H11" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="I11" t="str">
-        <v>23BSFT102</v>
-      </c>
-      <c r="J11" t="str">
-        <v>April - 2026</v>
-      </c>
-      <c r="K11" t="str">
-        <v>2026-05-04</v>
-      </c>
-      <c r="L11" t="str">
-        <v>IV</v>
-      </c>
-      <c r="M11" t="str">
-        <v>GCBSFT00002</v>
-      </c>
-      <c r="N11" t="str">
-        <v>CORE COURSE</v>
-      </c>
-      <c r="O11" t="str">
-        <v>THEORY</v>
-      </c>
-      <c r="P11">
-        <v>1</v>
-      </c>
-      <c r="Q11" t="str">
-        <v>SUB102</v>
-      </c>
-      <c r="R11" t="str">
-        <v>Introduction to Subject Two</v>
-      </c>
-      <c r="S11">
-        <v>4</v>
-      </c>
-      <c r="T11">
-        <v>4</v>
-      </c>
-      <c r="U11">
-        <v>35.2</v>
-      </c>
-      <c r="V11">
-        <v>52.8</v>
-      </c>
-      <c r="W11" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="X11" t="str">
-        <v>A+</v>
-      </c>
-      <c r="Y11">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>23bsft102@gcu.edu.in</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Rahul Krishnan</v>
-      </c>
-      <c r="D12" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Garden City University</v>
-      </c>
-      <c r="F12" t="str">
-        <v>SCHOOL OF SCIENCES</v>
-      </c>
-      <c r="G12" t="str">
-        <v>Bachelor of Science Food Science and Technology</v>
-      </c>
-      <c r="H12" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="I12" t="str">
-        <v>23BSFT102</v>
-      </c>
-      <c r="J12" t="str">
-        <v>April - 2026</v>
-      </c>
-      <c r="K12" t="str">
-        <v>2026-05-04</v>
-      </c>
-      <c r="L12" t="str">
-        <v>IV</v>
-      </c>
-      <c r="M12" t="str">
-        <v>GCBSFT00002</v>
-      </c>
-      <c r="N12" t="str">
-        <v>CORE COURSE</v>
-      </c>
-      <c r="O12" t="str">
-        <v>PRACTICAL</v>
-      </c>
-      <c r="P12">
-        <v>1</v>
-      </c>
-      <c r="Q12" t="str">
-        <v>SUB103P</v>
-      </c>
-      <c r="R12" t="str">
-        <v>Practical Lab One</v>
-      </c>
-      <c r="S12">
-        <v>4</v>
-      </c>
-      <c r="T12">
-        <v>4</v>
-      </c>
-      <c r="U12">
-        <v>38</v>
-      </c>
-      <c r="V12">
-        <v>57</v>
-      </c>
-      <c r="W12" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="X12" t="str">
-        <v>O</v>
-      </c>
-      <c r="Y12">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>23bsft102@gcu.edu.in</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Rahul Krishnan</v>
-      </c>
-      <c r="D13" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Garden City University</v>
-      </c>
-      <c r="F13" t="str">
-        <v>SCHOOL OF SCIENCES</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Bachelor of Science Food Science and Technology</v>
-      </c>
-      <c r="H13" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="I13" t="str">
-        <v>23BSFT102</v>
-      </c>
-      <c r="J13" t="str">
-        <v>April - 2026</v>
-      </c>
-      <c r="K13" t="str">
-        <v>2026-05-04</v>
-      </c>
-      <c r="L13" t="str">
-        <v>IV</v>
-      </c>
-      <c r="M13" t="str">
-        <v>GCBSFT00002</v>
-      </c>
-      <c r="N13" t="str">
-        <v>CORE COURSE</v>
-      </c>
-      <c r="O13" t="str">
-        <v>THEORY</v>
-      </c>
-      <c r="P13">
-        <v>1</v>
-      </c>
-      <c r="Q13" t="str">
-        <v>SUB104</v>
-      </c>
-      <c r="R13" t="str">
-        <v>Advanced Subject Four</v>
-      </c>
-      <c r="S13">
-        <v>4</v>
-      </c>
-      <c r="T13">
-        <v>4</v>
-      </c>
-      <c r="U13">
-        <v>27.200000000000003</v>
-      </c>
-      <c r="V13">
-        <v>40.8</v>
-      </c>
-      <c r="W13" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="X13" t="str">
-        <v>B+</v>
-      </c>
-      <c r="Y13">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>23bsft102@gcu.edu.in</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Rahul Krishnan</v>
-      </c>
-      <c r="D14" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Garden City University</v>
-      </c>
-      <c r="F14" t="str">
-        <v>SCHOOL OF SCIENCES</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Bachelor of Science Food Science and Technology</v>
-      </c>
-      <c r="H14" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="I14" t="str">
-        <v>23BSFT102</v>
-      </c>
-      <c r="J14" t="str">
-        <v>December - 2026</v>
-      </c>
-      <c r="K14" t="str">
-        <v>2026-05-04</v>
-      </c>
-      <c r="L14" t="str">
-        <v>V</v>
-      </c>
-      <c r="M14" t="str">
-        <v>GCBSFT00002</v>
-      </c>
-      <c r="N14" t="str">
-        <v>CORE COURSE</v>
-      </c>
-      <c r="O14" t="str">
-        <v>THEORY</v>
-      </c>
-      <c r="P14">
-        <v>1</v>
-      </c>
-      <c r="Q14" t="str">
-        <v>SUB101</v>
-      </c>
-      <c r="R14" t="str">
-        <v>Introduction to Subject One</v>
-      </c>
-      <c r="S14">
-        <v>4</v>
-      </c>
-      <c r="T14">
-        <v>4</v>
-      </c>
-      <c r="U14">
-        <v>30</v>
-      </c>
-      <c r="V14">
-        <v>45</v>
-      </c>
-      <c r="W14" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="X14" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y14">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>23bsft102@gcu.edu.in</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Rahul Krishnan</v>
-      </c>
-      <c r="D15" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Garden City University</v>
-      </c>
-      <c r="F15" t="str">
-        <v>SCHOOL OF SCIENCES</v>
-      </c>
-      <c r="G15" t="str">
-        <v>Bachelor of Science Food Science and Technology</v>
-      </c>
-      <c r="H15" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="I15" t="str">
-        <v>23BSFT102</v>
-      </c>
-      <c r="J15" t="str">
-        <v>December - 2026</v>
-      </c>
-      <c r="K15" t="str">
-        <v>2026-05-04</v>
-      </c>
-      <c r="L15" t="str">
-        <v>V</v>
-      </c>
-      <c r="M15" t="str">
-        <v>GCBSFT00002</v>
-      </c>
-      <c r="N15" t="str">
-        <v>CORE COURSE</v>
-      </c>
-      <c r="O15" t="str">
-        <v>THEORY</v>
-      </c>
-      <c r="P15">
-        <v>1</v>
-      </c>
-      <c r="Q15" t="str">
-        <v>SUB102</v>
-      </c>
-      <c r="R15" t="str">
-        <v>Introduction to Subject Two</v>
-      </c>
-      <c r="S15">
-        <v>4</v>
-      </c>
-      <c r="T15">
-        <v>4</v>
-      </c>
-      <c r="U15">
-        <v>35.2</v>
-      </c>
-      <c r="V15">
-        <v>52.8</v>
-      </c>
-      <c r="W15" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="X15" t="str">
-        <v>A+</v>
-      </c>
-      <c r="Y15">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>23bsft102@gcu.edu.in</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Rahul Krishnan</v>
-      </c>
-      <c r="D16" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Garden City University</v>
-      </c>
-      <c r="F16" t="str">
-        <v>SCHOOL OF SCIENCES</v>
-      </c>
-      <c r="G16" t="str">
-        <v>Bachelor of Science Food Science and Technology</v>
-      </c>
-      <c r="H16" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="I16" t="str">
-        <v>23BSFT102</v>
-      </c>
-      <c r="J16" t="str">
-        <v>December - 2026</v>
-      </c>
-      <c r="K16" t="str">
-        <v>2026-05-04</v>
-      </c>
-      <c r="L16" t="str">
-        <v>V</v>
-      </c>
-      <c r="M16" t="str">
-        <v>GCBSFT00002</v>
-      </c>
-      <c r="N16" t="str">
-        <v>CORE COURSE</v>
-      </c>
-      <c r="O16" t="str">
-        <v>PRACTICAL</v>
-      </c>
-      <c r="P16">
-        <v>1</v>
-      </c>
-      <c r="Q16" t="str">
-        <v>SUB103P</v>
-      </c>
-      <c r="R16" t="str">
-        <v>Practical Lab One</v>
-      </c>
-      <c r="S16">
-        <v>4</v>
-      </c>
-      <c r="T16">
-        <v>4</v>
-      </c>
-      <c r="U16">
-        <v>38</v>
-      </c>
-      <c r="V16">
-        <v>57</v>
-      </c>
-      <c r="W16" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="X16" t="str">
-        <v>O</v>
-      </c>
-      <c r="Y16">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="str">
-        <v>23bsft102@gcu.edu.in</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Rahul Krishnan</v>
-      </c>
-      <c r="D17" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Garden City University</v>
-      </c>
-      <c r="F17" t="str">
-        <v>SCHOOL OF SCIENCES</v>
-      </c>
-      <c r="G17" t="str">
-        <v>Bachelor of Science Food Science and Technology</v>
-      </c>
-      <c r="H17" t="str">
-        <v>BSFT</v>
-      </c>
-      <c r="I17" t="str">
-        <v>23BSFT102</v>
-      </c>
-      <c r="J17" t="str">
-        <v>December - 2026</v>
-      </c>
-      <c r="K17" t="str">
-        <v>2026-05-04</v>
-      </c>
-      <c r="L17" t="str">
-        <v>V</v>
-      </c>
-      <c r="M17" t="str">
-        <v>GCBSFT00002</v>
-      </c>
-      <c r="N17" t="str">
-        <v>CORE COURSE</v>
-      </c>
-      <c r="O17" t="str">
-        <v>THEORY</v>
-      </c>
-      <c r="P17">
-        <v>1</v>
-      </c>
-      <c r="Q17" t="str">
-        <v>SUB104</v>
-      </c>
-      <c r="R17" t="str">
-        <v>Advanced Subject Four</v>
-      </c>
-      <c r="S17">
-        <v>4</v>
-      </c>
-      <c r="T17">
-        <v>4</v>
-      </c>
-      <c r="U17">
-        <v>27.200000000000003</v>
-      </c>
-      <c r="V17">
-        <v>40.8</v>
-      </c>
-      <c r="W17" t="str">
-        <v>PASS</v>
-      </c>
-      <c r="X17" t="str">
-        <v>B+</v>
-      </c>
-      <c r="Y17">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>